<commit_message>
Fix Week 4 booked hours
</commit_message>
<xml_diff>
--- a/Documentation/Week 4/Booked Hours/Booked_Hours_Murphy.xlsx
+++ b/Documentation/Week 4/Booked Hours/Booked_Hours_Murphy.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr date1904="1"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11960" tabRatio="500"/>
+    <workbookView windowWidth="24200" windowHeight="11980" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="15">
   <si>
     <r>
       <rPr>
@@ -74,6 +74,12 @@
   </si>
   <si>
     <t>Attend weekly group meetings with client</t>
+  </si>
+  <si>
+    <t>Download the Ubuntu 22.04.5 and set up all dependencies</t>
+  </si>
+  <si>
+    <t>Understand the entire process and details of gesture recognition</t>
   </si>
 </sst>
 </file>
@@ -1391,7 +1397,7 @@
     <col min="3" max="3" width="8.1640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="9.3359375" style="1" customWidth="1"/>
     <col min="5" max="5" width="8.8359375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="46.5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="51.859375" style="1" customWidth="1"/>
     <col min="7" max="7" width="9.3359375" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" style="1"/>
     <col min="9" max="9" width="10.6640625" style="1" hidden="1" customWidth="1"/>
@@ -1674,76 +1680,132 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="11" spans="2:9">
-      <c r="B11" s="13"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="12"/>
-      <c r="G11" s="19" t="str">
+    <row r="11" spans="1:9">
+      <c r="A11" s="1">
+        <v>4</v>
+      </c>
+      <c r="B11" s="10">
+        <v>44783</v>
+      </c>
+      <c r="C11" s="12">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="D11" s="10">
+        <v>44783</v>
+      </c>
+      <c r="E11" s="12">
+        <v>0.75</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="19">
         <f t="shared" si="0"/>
-        <v> </v>
-      </c>
-      <c r="H11" s="1" t="str">
+        <v>2.00000000005821</v>
+      </c>
+      <c r="H11" s="1">
         <f t="shared" si="2"/>
-        <v> </v>
+        <v>11.4999999997672</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9">
-      <c r="B12" s="13"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="12"/>
-      <c r="G12" s="19" t="str">
+        <v>2.00000000005821</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="1">
+        <v>4</v>
+      </c>
+      <c r="B12" s="10">
+        <v>44784</v>
+      </c>
+      <c r="C12" s="12">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="D12" s="10">
+        <v>44784</v>
+      </c>
+      <c r="E12" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="19">
         <f t="shared" si="0"/>
-        <v> </v>
-      </c>
-      <c r="H12" s="1" t="str">
+        <v>0.999999999941792</v>
+      </c>
+      <c r="H12" s="1">
         <f t="shared" si="2"/>
-        <v> </v>
+        <v>12.499999999709</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9">
-      <c r="B13" s="13"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="12"/>
-      <c r="G13" s="19" t="str">
+        <v>0.999999999941792</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="1">
+        <v>4</v>
+      </c>
+      <c r="B13" s="10">
+        <v>44784</v>
+      </c>
+      <c r="C13" s="12">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D13" s="10">
+        <v>44784</v>
+      </c>
+      <c r="E13" s="12">
+        <v>0.5625</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="19">
         <f t="shared" si="0"/>
-        <v> </v>
-      </c>
-      <c r="H13" s="1" t="str">
+        <v>0.500000000058208</v>
+      </c>
+      <c r="H13" s="1">
         <f t="shared" si="2"/>
-        <v> </v>
+        <v>12.9999999997672</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:9">
-      <c r="B14" s="13"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="12"/>
-      <c r="G14" s="19" t="str">
+        <v>0.500000000058208</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="1">
+        <v>4</v>
+      </c>
+      <c r="B14" s="10">
+        <v>44786</v>
+      </c>
+      <c r="C14" s="12">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D14" s="10">
+        <v>44786</v>
+      </c>
+      <c r="E14" s="12">
+        <v>0.604166666666667</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="19">
         <f t="shared" si="0"/>
-        <v> </v>
-      </c>
-      <c r="H14" s="1" t="str">
+        <v>1.5</v>
+      </c>
+      <c r="H14" s="1">
         <f t="shared" si="2"/>
-        <v> </v>
+        <v>14.4999999997672</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="15" spans="2:9">

</xml_diff>